<commit_message>
corrected hig file 2025
</commit_message>
<xml_diff>
--- a/data/hig/original_data/HIG_APC_2025.xlsx
+++ b/data/hig/original_data/HIG_APC_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="I:\Forskarstöd\Open access\APC kostnader\Open APC Sweden\2025\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F84C58A-2AF1-4772-9420-073182DEE445}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58CCF3C9-DA87-4FB4-9C9B-FED001D256D3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="25620" yWindow="0" windowWidth="25980" windowHeight="20880" xr2:uid="{A6F00635-5C01-4C60-BDF9-17EF2738987C}"/>
+    <workbookView xWindow="25710" yWindow="0" windowWidth="25980" windowHeight="20970" xr2:uid="{A6F00635-5C01-4C60-BDF9-17EF2738987C}"/>
   </bookViews>
   <sheets>
     <sheet name="HIG_APC_2025" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="42">
   <si>
     <t>institution</t>
   </si>
@@ -86,9 +86,6 @@
     <t>10.1515/rams-2024-0076</t>
   </si>
   <si>
-    <t>10.1061/JUPDDM/UPENG-5334</t>
-  </si>
-  <si>
     <t>10.3390/soc15010017</t>
   </si>
   <si>
@@ -143,30 +140,6 @@
     <t xml:space="preserve">hig </t>
   </si>
   <si>
-    <t>Inderscience</t>
-  </si>
-  <si>
-    <t>International Journal of Management and Enterprise Development</t>
-  </si>
-  <si>
-    <t>1468-4330</t>
-  </si>
-  <si>
-    <t>1741-8127</t>
-  </si>
-  <si>
-    <t>SIPISS- Edizioni FS Publishers</t>
-  </si>
-  <si>
-    <t>Journal of Health and Social Sciences</t>
-  </si>
-  <si>
-    <t>2499-2240</t>
-  </si>
-  <si>
-    <t>2499-5886</t>
-  </si>
-  <si>
     <t>10.3390/en18215572</t>
   </si>
   <si>
@@ -180,18 +153,34 @@
   </si>
   <si>
     <t>10.3390/admsci15020056</t>
+  </si>
+  <si>
+    <t>10.1504/IJMED.2026.151258</t>
+  </si>
+  <si>
+    <t>10.19204/2025/DSNQ8</t>
+  </si>
+  <si>
+    <t>10.1061/JUPDDM.UPENG-5334</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
     <font>
       <sz val="11"/>
@@ -221,10 +210,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="1" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="1" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -667,8 +657,8 @@
       <c r="C6" s="2">
         <v>28160.52</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>16</v>
+      <c r="D6" s="3" t="s">
+        <v>41</v>
       </c>
       <c r="E6" s="1" t="b">
         <v>1</v>
@@ -685,7 +675,7 @@
         <v>13541</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E7" s="1" t="b">
         <v>0</v>
@@ -702,7 +692,7 @@
         <v>23212</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="E8" s="1" t="b">
         <v>0</v>
@@ -719,7 +709,7 @@
         <v>24381.34</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="E9" s="1" t="b">
         <v>0</v>
@@ -736,7 +726,7 @@
         <v>12964.06</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>47</v>
+        <v>38</v>
       </c>
       <c r="E10" s="1" t="b">
         <v>0</v>
@@ -753,7 +743,7 @@
         <v>24334.42</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E11" s="1" t="b">
         <v>1</v>
@@ -770,7 +760,7 @@
         <v>35108.800000000003</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="E12" s="1" t="b">
         <v>0</v>
@@ -787,7 +777,7 @@
         <v>22786</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="E13" s="1" t="b">
         <v>0</v>
@@ -804,7 +794,7 @@
         <v>18404</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="E14" s="1" t="b">
         <v>0</v>
@@ -821,7 +811,7 @@
         <v>21033</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E15" s="1" t="b">
         <v>0</v>
@@ -838,13 +828,13 @@
         <v>21969</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E16" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="17" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" s="1" t="s">
         <v>11</v>
       </c>
@@ -855,13 +845,13 @@
         <v>13843.44</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E17" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
         <v>11</v>
       </c>
@@ -872,13 +862,13 @@
         <v>8200.1299999999992</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E18" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
         <v>11</v>
       </c>
@@ -889,13 +879,13 @@
         <v>17093.61</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E19" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" s="1" t="s">
         <v>11</v>
       </c>
@@ -906,13 +896,13 @@
         <v>22845.52</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="E20" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" s="1" t="s">
         <v>11</v>
       </c>
@@ -923,13 +913,13 @@
         <v>27592.5</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="E21" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
         <v>11</v>
       </c>
@@ -940,13 +930,13 @@
         <v>22060</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="E22" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="23" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" s="1" t="s">
         <v>11</v>
       </c>
@@ -957,13 +947,13 @@
         <v>12387.15</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="E23" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
         <v>11</v>
       </c>
@@ -974,15 +964,15 @@
         <v>39009.03</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E24" s="1" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B25" s="1">
         <v>2025</v>
@@ -990,23 +980,14 @@
       <c r="C25" s="2">
         <v>21880</v>
       </c>
+      <c r="D25" s="1" t="s">
+        <v>39</v>
+      </c>
       <c r="E25" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="F25" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="G25" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="I25" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="J25" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
         <v>11</v>
       </c>
@@ -1016,23 +997,14 @@
       <c r="C26" s="2">
         <v>4912</v>
       </c>
+      <c r="D26" s="1" t="s">
+        <v>40</v>
+      </c>
       <c r="E26" s="1" t="b">
         <v>0</v>
       </c>
-      <c r="F26" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="I26" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="J26" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="27" spans="1:10" x14ac:dyDescent="0.25">
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
         <v>11</v>
       </c>
@@ -1043,13 +1015,13 @@
         <v>23084</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>43</v>
+        <v>34</v>
       </c>
       <c r="E27" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
         <v>11</v>
       </c>
@@ -1060,13 +1032,13 @@
         <v>12391</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
       <c r="E28" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
         <v>11</v>
       </c>
@@ -1077,13 +1049,13 @@
         <v>23697</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E29" s="1" t="b">
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:10" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
         <v>11</v>
       </c>
@@ -1094,7 +1066,7 @@
         <v>15798</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>46</v>
+        <v>37</v>
       </c>
       <c r="E30" s="1" t="b">
         <v>0</v>

</xml_diff>